<commit_message>
3-8 changes (perovskite and lab data analysis)
</commit_message>
<xml_diff>
--- a/3_8_advanced_prompting/perovskite_data.xlsx
+++ b/3_8_advanced_prompting/perovskite_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,15 +436,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>La0.7Ba0.3Mn03</t>
+          <t>La0.7Sr0.3MnO3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ba0.5Sr0.5TiO3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>La0.7Ba0.3MnO3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>1120</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>3</t>
         </is>

</xml_diff>